<commit_message>
Mejora UI, separa comentario causal RAG y refactoriza evaluacion
</commit_message>
<xml_diff>
--- a/data/sample/mineria_hidrocarburos_202602.xlsx
+++ b/data/sample/mineria_hidrocarburos_202602.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\JC2026\AGENTE_REPORTES\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\03 PROYECTOS\agente-reportes-economicos\data\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CD741CD-A48B-40C6-B669-0CA786EB279A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4932F1B9-C009-4119-B324-807CF65FCCA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8EFFB3D2-6B7E-4748-B1C0-079B24D71080}"/>
   </bookViews>
@@ -29,6 +29,9 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -84,9 +87,6 @@
     <t>Minería e Hidrocarburos</t>
   </si>
   <si>
-    <t>Minería Metálica</t>
-  </si>
-  <si>
     <t>variacion_acumulada</t>
   </si>
   <si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>sector</t>
+  </si>
+  <si>
+    <t>Minería metálica</t>
   </si>
 </sst>
 </file>
@@ -179,9 +182,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -219,7 +222,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -325,7 +328,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -467,7 +470,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -492,10 +495,10 @@
         <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D1" t="s">
         <v>13</v>
@@ -504,10 +507,10 @@
         <v>14</v>
       </c>
       <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
         <v>17</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -515,7 +518,7 @@
         <v>202602</v>
       </c>
       <c r="B2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -538,10 +541,10 @@
         <v>202602</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D3">
         <v>0.12955578925914324</v>
@@ -561,7 +564,7 @@
         <v>202602</v>
       </c>
       <c r="B4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>0</v>
@@ -584,22 +587,22 @@
         <v>202602</v>
       </c>
       <c r="B5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D5">
-        <v>1.4843341278130566</v>
+        <v>0.14748056044324187</v>
       </c>
       <c r="E5">
-        <v>4.9664771230967117E-2</v>
+        <v>1.4916809152760566E-2</v>
       </c>
       <c r="F5">
-        <v>1.3527422061113725</v>
+        <v>2.1622458149435033</v>
       </c>
       <c r="G5">
-        <v>4.6146126225767616E-2</v>
+        <v>0.23154815513860164</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -607,22 +610,22 @@
         <v>202602</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D6">
-        <v>0.14748056044324187</v>
+        <v>-1.055253007700415</v>
       </c>
       <c r="E6">
-        <v>1.4916809152760566E-2</v>
+        <v>-9.6706844526037394E-2</v>
       </c>
       <c r="F6">
-        <v>2.1622458149435033</v>
+        <v>6.1281187741898151</v>
       </c>
       <c r="G6">
-        <v>0.23154815513860164</v>
+        <v>0.51889812829647997</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -630,22 +633,22 @@
         <v>202602</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7">
-        <v>0.50930772851327788</v>
+        <v>-2.6533136934814081</v>
       </c>
       <c r="E7">
-        <v>2.1593428340119796E-3</v>
+        <v>-0.13401349833869985</v>
       </c>
       <c r="F7">
-        <v>2.2215923647360398</v>
+        <v>0.77155033893954794</v>
       </c>
       <c r="G7">
-        <v>9.3536049373758538E-3</v>
+        <v>3.7581464652946039E-2</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -653,22 +656,22 @@
         <v>202602</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="D8">
-        <v>-1.055253007700415</v>
+        <v>-9.6334257257778972</v>
       </c>
       <c r="E8">
-        <v>-9.6706844526037394E-2</v>
+        <v>-0.8442081919193527</v>
       </c>
       <c r="F8">
-        <v>6.1281187741898151</v>
+        <v>-6.9367306693909256</v>
       </c>
       <c r="G8">
-        <v>0.51889812829647997</v>
+        <v>-0.59157124576299813</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -676,7 +679,7 @@
         <v>202602</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>6</v>
@@ -699,22 +702,22 @@
         <v>202602</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D10">
-        <v>-2.6533136934814081</v>
+        <v>1.4843341278130566</v>
       </c>
       <c r="E10">
-        <v>-0.13401349833869985</v>
+        <v>4.9664771230967117E-2</v>
       </c>
       <c r="F10">
-        <v>0.77155033893954794</v>
+        <v>1.3527422061113725</v>
       </c>
       <c r="G10">
-        <v>3.7581464652946039E-2</v>
+        <v>4.6146126225767616E-2</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -722,22 +725,22 @@
         <v>202602</v>
       </c>
       <c r="B11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D11">
-        <v>-9.6334257257778972</v>
+        <v>0.50930772851327788</v>
       </c>
       <c r="E11">
-        <v>-0.8442081919193527</v>
+        <v>2.1593428340119796E-3</v>
       </c>
       <c r="F11">
-        <v>-6.9367306693909256</v>
+        <v>2.2215923647360398</v>
       </c>
       <c r="G11">
-        <v>-0.59157124576299813</v>
+        <v>9.3536049373758538E-3</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -745,7 +748,7 @@
         <v>202602</v>
       </c>
       <c r="B12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
@@ -768,7 +771,7 @@
         <v>202602</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>9</v>
@@ -791,7 +794,7 @@
         <v>202602</v>
       </c>
       <c r="B14" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>10</v>
@@ -814,7 +817,7 @@
         <v>202602</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>11</v>

</xml_diff>